<commit_message>
Polish call cost model spreadsheet: cleaner green theme, grouped sections, zebra rows, framed total
</commit_message>
<xml_diff>
--- a/call-cost-model.xlsx
+++ b/call-cost-model.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Call Cost Model" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Cost Model" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,7 +20,7 @@
     <numFmt numFmtId="164" formatCode="$0.000"/>
     <numFmt numFmtId="165" formatCode="$0.00"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -29,61 +29,81 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Arial"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="14"/>
-    </font>
-    <font>
+      <sz val="18"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
       <b val="1"/>
-    </font>
-    <font>
+      <color rgb="00475569"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
       <b val="1"/>
-      <color rgb="001D4ED8"/>
-    </font>
-    <font>
+      <color rgb="00065F46"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Arial"/>
       <i val="1"/>
-    </font>
-    <font>
+      <color rgb="00475569"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00065F46"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="000F172A"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00475569"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="000F172A"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="0015803D"/>
+      <sz val="10"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="000C0C12"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00DBEAFE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FEF9C3"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="001F2937"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E5E7EB"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FEF3C7"/>
-      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -95,8 +115,33 @@
         <fgColor rgb="00DCFCE7"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F8FAFC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000F172A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00ECFDF5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F1F5F9"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="5">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -104,115 +149,84 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="00CBD5E1"/>
-      </left>
-      <right style="thin">
-        <color rgb="00CBD5E1"/>
-      </right>
-      <top style="thin">
-        <color rgb="00CBD5E1"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00CBD5E1"/>
-      </bottom>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="00CBD5E1"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="00CBD5E1"/>
-      </right>
-      <top style="thin">
-        <color rgb="00CBD5E1"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="00CBD5E1"/>
-      </right>
-      <top style="thin">
-        <color rgb="00CBD5E1"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00CBD5E1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="12" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="12" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="12" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="12" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="1" fontId="12" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -583,549 +597,561 @@
   <dimension ref="A1:E36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="46" customWidth="1" min="1" max="1"/>
-    <col width="68" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="31" customWidth="1" min="1" max="1"/>
+    <col width="56" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1" ht="24" customHeight="1">
+    <row r="1" ht="36" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Cost to Serve One Call  —  by Call Type</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
+          <t>📞  Cost to Serve One Call</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Select call type ▶</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="inlineStr">
+          <t>Pick a call type below — every number updates live. Columns = seconds talking to a human.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="24" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>CALL TYPE</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>VOICE (voice only tree - CVS)</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="4">
-        <f>"This type reaches a human in about "&amp;$B$25&amp;" seconds. Each column then adds that many seconds of talking to the person."</f>
-        <v/>
-      </c>
-    </row>
     <row r="5">
-      <c r="A5" s="5" t="inlineStr">
-        <is>
-          <t>Service</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>What it is doing</t>
-        </is>
-      </c>
-      <c r="C5" s="6" t="inlineStr">
-        <is>
-          <t>30 sec talk</t>
-        </is>
-      </c>
-      <c r="D5" s="6" t="inlineStr">
-        <is>
-          <t>45 sec talk</t>
-        </is>
-      </c>
-      <c r="E5" s="6" t="inlineStr">
-        <is>
-          <t>60 sec talk</t>
-        </is>
+      <c r="A5" s="5">
+        <f>"ℹ︎  This type reaches a human in about "&amp;$B$25&amp;" seconds, then talks for the time in each column."</f>
+        <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="inlineStr">
-        <is>
-          <t>①  REACH THE HUMAN   (same cost no matter how long you talk)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="8" t="inlineStr">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>①   REACH THE HUMAN     ·  same cost no matter how long you talk</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="34" customHeight="1">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t>Twilio Speech-to-Text</t>
         </is>
       </c>
-      <c r="B7" s="9" t="inlineStr">
-        <is>
-          <t>The cheap navigator's EARS. Transcribes the store's spoken menu so Haiku can read it.</t>
-        </is>
-      </c>
-      <c r="C7" s="10">
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>The cheap navigator's EARS — transcribes the store's spoken menu so Haiku can read it.</t>
+        </is>
+      </c>
+      <c r="C7" s="9">
         <f>IF($B$35=1,$B$25*$B$27/60,0)</f>
         <v/>
       </c>
-      <c r="D7" s="10">
+      <c r="D7" s="9">
         <f>IF($B$35=1,$B$25*$B$27/60,0)</f>
         <v/>
       </c>
-      <c r="E7" s="10">
+      <c r="E7" s="9">
         <f>IF($B$35=1,$B$25*$B$27/60,0)</f>
         <v/>
       </c>
     </row>
-    <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="8" t="inlineStr">
+    <row r="8" ht="34" customHeight="1">
+      <c r="A8" s="10" t="inlineStr">
         <is>
           <t>Claude Haiku</t>
         </is>
       </c>
-      <c r="B8" s="9" t="inlineStr">
-        <is>
-          <t>The cheap navigator's BRAIN. Reads the menu and picks the word to say (no, front, general).</t>
-        </is>
-      </c>
-      <c r="C8" s="10">
+      <c r="B8" s="11" t="inlineStr">
+        <is>
+          <t>The cheap navigator's BRAIN — reads the menu and picks the word to say (no, front, general).</t>
+        </is>
+      </c>
+      <c r="C8" s="12">
         <f>IF($B$35=1,$B$28,0)</f>
         <v/>
       </c>
-      <c r="D8" s="10">
+      <c r="D8" s="12">
         <f>IF($B$35=1,$B$28,0)</f>
         <v/>
       </c>
-      <c r="E8" s="10">
+      <c r="E8" s="12">
         <f>IF($B$35=1,$B$28,0)</f>
         <v/>
       </c>
     </row>
-    <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="8" t="inlineStr">
+    <row r="9" ht="34" customHeight="1">
+      <c r="A9" s="7" t="inlineStr">
         <is>
           <t>Cheap Text-to-Speech</t>
         </is>
       </c>
-      <c r="B9" s="9" t="inlineStr">
-        <is>
-          <t>The cheap navigator's MOUTH. Speaks that word into the menu to move it forward.</t>
-        </is>
-      </c>
-      <c r="C9" s="10">
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>The cheap navigator's MOUTH — speaks that word into the menu to move it forward.</t>
+        </is>
+      </c>
+      <c r="C9" s="9">
         <f>IF($B$35=1,$B$29,0)</f>
         <v/>
       </c>
-      <c r="D9" s="10">
+      <c r="D9" s="9">
         <f>IF($B$35=1,$B$29,0)</f>
         <v/>
       </c>
-      <c r="E9" s="10">
+      <c r="E9" s="9">
         <f>IF($B$35=1,$B$29,0)</f>
         <v/>
       </c>
     </row>
-    <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="8" t="inlineStr">
+    <row r="10" ht="34" customHeight="1">
+      <c r="A10" s="10" t="inlineStr">
         <is>
           <t>Our bridge (button presses)</t>
         </is>
       </c>
-      <c r="B10" s="9" t="inlineStr">
-        <is>
-          <t>Keypad stores only: our server plays the keypad tones at the right time. No AI, basically free.</t>
-        </is>
-      </c>
-      <c r="C10" s="10">
+      <c r="B10" s="11" t="inlineStr">
+        <is>
+          <t>Keypad stores only — our server plays the keypad tones at the right time. No AI, basically free.</t>
+        </is>
+      </c>
+      <c r="C10" s="12">
         <f>0</f>
         <v/>
       </c>
-      <c r="D10" s="10">
+      <c r="D10" s="12">
         <f>0</f>
         <v/>
       </c>
-      <c r="E10" s="10">
+      <c r="E10" s="12">
         <f>0</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="11" t="inlineStr">
-        <is>
-          <t>Subtotal — reach the human</t>
-        </is>
-      </c>
-      <c r="B11" s="12" t="n"/>
-      <c r="C11" s="13">
+      <c r="A11" s="13" t="inlineStr">
+        <is>
+          <t>Subtotal to reach the human</t>
+        </is>
+      </c>
+      <c r="C11" s="14">
         <f>SUM(C7:C10)</f>
         <v/>
       </c>
-      <c r="D11" s="13">
+      <c r="D11" s="14">
         <f>SUM(D7:D10)</f>
         <v/>
       </c>
-      <c r="E11" s="13">
+      <c r="E11" s="14">
         <f>SUM(E7:E10)</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="7" t="inlineStr">
-        <is>
-          <t>②  TALK TO THE HUMAN   (this is what grows across the columns)</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="30" customHeight="1">
-      <c r="A13" s="8" t="inlineStr">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>②   TALK TO THE HUMAN     ·  this is what grows across the columns</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="34" customHeight="1">
+      <c r="A13" s="7" t="inlineStr">
         <is>
           <t>ElevenLabs Conversational AI</t>
         </is>
       </c>
-      <c r="B13" s="9" t="inlineStr">
+      <c r="B13" s="8" t="inlineStr">
         <is>
           <t>Premium voice engine for the human chat: speech-to-text, the voice, and turn-taking. Billed only while connected to the person.</t>
         </is>
       </c>
-      <c r="C13" s="10">
+      <c r="C13" s="9">
         <f>30*$B$30/60</f>
         <v/>
       </c>
-      <c r="D13" s="10">
+      <c r="D13" s="9">
         <f>45*$B$30/60</f>
         <v/>
       </c>
-      <c r="E13" s="10">
+      <c r="E13" s="9">
         <f>60*$B$30/60</f>
         <v/>
       </c>
     </row>
-    <row r="14" ht="30" customHeight="1">
-      <c r="A14" s="8" t="inlineStr">
+    <row r="14" ht="34" customHeight="1">
+      <c r="A14" s="10" t="inlineStr">
         <is>
           <t>Claude Sonnet 4.6</t>
         </is>
       </c>
-      <c r="B14" s="9" t="inlineStr">
-        <is>
-          <t>The smart brain during the human conversation. Understands the clerk and answers naturally.</t>
-        </is>
-      </c>
-      <c r="C14" s="10">
+      <c r="B14" s="11" t="inlineStr">
+        <is>
+          <t>The smart brain during the human conversation — understands the clerk and answers naturally.</t>
+        </is>
+      </c>
+      <c r="C14" s="12">
         <f>30*$B$31/60</f>
         <v/>
       </c>
-      <c r="D14" s="10">
+      <c r="D14" s="12">
         <f>45*$B$31/60</f>
         <v/>
       </c>
-      <c r="E14" s="10">
+      <c r="E14" s="12">
         <f>60*$B$31/60</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="11" t="inlineStr">
-        <is>
-          <t>Subtotal — talk to the human</t>
-        </is>
-      </c>
-      <c r="B15" s="12" t="n"/>
-      <c r="C15" s="13">
+      <c r="A15" s="13" t="inlineStr">
+        <is>
+          <t>Subtotal to talk to the human</t>
+        </is>
+      </c>
+      <c r="C15" s="14">
         <f>SUM(C13:C14)</f>
         <v/>
       </c>
-      <c r="D15" s="13">
+      <c r="D15" s="14">
         <f>SUM(D13:D14)</f>
         <v/>
       </c>
-      <c r="E15" s="13">
+      <c r="E15" s="14">
         <f>SUM(E13:E14)</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="7" t="inlineStr">
-        <is>
-          <t>③  THE LINE   (runs the whole call)</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="30" customHeight="1">
-      <c r="A17" s="8" t="inlineStr">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>③   THE LINE     ·  runs the whole call</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="34" customHeight="1">
+      <c r="A17" s="7" t="inlineStr">
         <is>
           <t>Twilio Voice</t>
         </is>
       </c>
-      <c r="B17" s="9" t="inlineStr">
-        <is>
-          <t>The phone line: dials the store, carries the audio both ways, shows your caller ID.</t>
-        </is>
-      </c>
-      <c r="C17" s="10">
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>The phone line — dials the store, carries the audio both ways, shows your caller ID.</t>
+        </is>
+      </c>
+      <c r="C17" s="9">
         <f>($B$25+30)*$B$26/60</f>
         <v/>
       </c>
-      <c r="D17" s="10">
+      <c r="D17" s="9">
         <f>($B$25+45)*$B$26/60</f>
         <v/>
       </c>
-      <c r="E17" s="10">
+      <c r="E17" s="9">
         <f>($B$25+60)*$B$26/60</f>
         <v/>
       </c>
     </row>
-    <row r="18" ht="30" customHeight="1">
-      <c r="A18" s="8" t="inlineStr">
+    <row r="18" ht="34" customHeight="1">
+      <c r="A18" s="10" t="inlineStr">
         <is>
           <t>Railway server</t>
         </is>
       </c>
-      <c r="B18" s="9" t="inlineStr">
+      <c r="B18" s="11" t="inlineStr">
         <is>
           <t>Our app that runs the call and bridges the audio.</t>
         </is>
       </c>
-      <c r="C18" s="10">
+      <c r="C18" s="12">
         <f>$B$32</f>
         <v/>
       </c>
-      <c r="D18" s="10">
+      <c r="D18" s="12">
         <f>$B$32</f>
         <v/>
       </c>
-      <c r="E18" s="10">
+      <c r="E18" s="12">
         <f>$B$32</f>
         <v/>
       </c>
     </row>
-    <row r="19" ht="30" customHeight="1">
-      <c r="A19" s="8" t="inlineStr">
+    <row r="19" ht="34" customHeight="1">
+      <c r="A19" s="7" t="inlineStr">
         <is>
           <t>Twilio number rental</t>
         </is>
       </c>
-      <c r="B19" s="9" t="inlineStr">
+      <c r="B19" s="8" t="inlineStr">
         <is>
           <t>Monthly cost of the phone number, spread across calls.</t>
         </is>
       </c>
-      <c r="C19" s="10">
+      <c r="C19" s="9">
         <f>$B$33</f>
         <v/>
       </c>
-      <c r="D19" s="10">
+      <c r="D19" s="9">
         <f>$B$33</f>
         <v/>
       </c>
-      <c r="E19" s="10">
+      <c r="E19" s="9">
         <f>$B$33</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="11" t="inlineStr">
-        <is>
-          <t>Subtotal — the line</t>
-        </is>
-      </c>
-      <c r="B20" s="12" t="n"/>
-      <c r="C20" s="13">
+      <c r="A20" s="13" t="inlineStr">
+        <is>
+          <t>Subtotal for the line</t>
+        </is>
+      </c>
+      <c r="C20" s="14">
         <f>SUM(C17:C19)</f>
         <v/>
       </c>
-      <c r="D20" s="13">
+      <c r="D20" s="14">
         <f>SUM(D17:D19)</f>
         <v/>
       </c>
-      <c r="E20" s="13">
+      <c r="E20" s="14">
         <f>SUM(E17:E19)</f>
         <v/>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="14" t="inlineStr">
+    <row r="21" ht="28" customHeight="1">
+      <c r="A21" s="15" t="inlineStr">
         <is>
           <t>TOTAL COST TO SERVE</t>
         </is>
       </c>
-      <c r="B21" s="12" t="n"/>
-      <c r="C21" s="15">
+      <c r="C21" s="16">
         <f>C11+C15+C20</f>
         <v/>
       </c>
-      <c r="D21" s="15">
+      <c r="D21" s="16">
         <f>D11+D15+D20</f>
         <v/>
       </c>
-      <c r="E21" s="15">
+      <c r="E21" s="16">
         <f>E11+E15+E20</f>
         <v/>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="16" t="inlineStr">
+    <row r="22" ht="22" customHeight="1">
+      <c r="A22" s="17" t="inlineStr">
         <is>
           <t>Your margin at the price below</t>
         </is>
       </c>
-      <c r="B22" s="12" t="n"/>
-      <c r="C22" s="17">
+      <c r="C22" s="18">
         <f>$B$34-C21</f>
         <v/>
       </c>
-      <c r="D22" s="17">
+      <c r="D22" s="18">
         <f>$B$34-D21</f>
         <v/>
       </c>
-      <c r="E22" s="17">
+      <c r="E22" s="18">
         <f>$B$34-E21</f>
         <v/>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="5" t="inlineStr">
-        <is>
-          <t>ASSUMPTIONS &amp; RATES   (edit any value and the whole table recalculates)</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="9" t="inlineStr">
-        <is>
-          <t>Reach-the-human seconds (set automatically by the type)</t>
-        </is>
-      </c>
-      <c r="B25" s="18">
+      <c r="A24" s="19" t="inlineStr">
+        <is>
+          <t>ASSUMPTIONS &amp; RATES   ·   edit any value and the whole table recalculates</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="22" customHeight="1">
+      <c r="A25" s="8" t="inlineStr">
+        <is>
+          <t>Reach-the-human seconds (auto-set by the type)</t>
+        </is>
+      </c>
+      <c r="B25" s="20">
         <f>IF(B2="VOICE (voice only tree - CVS)",30,IF(B2="KEYPAD (no voice tree - Walgreens)",20,5))</f>
         <v/>
       </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="9" t="inlineStr">
+      <c r="C25" s="21" t="n"/>
+      <c r="D25" s="21" t="n"/>
+      <c r="E25" s="21" t="n"/>
+    </row>
+    <row r="26" ht="22" customHeight="1">
+      <c r="A26" s="11" t="inlineStr">
         <is>
           <t>Twilio carrier, $ per minute</t>
         </is>
       </c>
-      <c r="B26" s="19" t="n">
+      <c r="B26" s="22" t="n">
         <v>0.014</v>
       </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="9" t="inlineStr">
+      <c r="C26" s="23" t="n"/>
+      <c r="D26" s="23" t="n"/>
+      <c r="E26" s="23" t="n"/>
+    </row>
+    <row r="27" ht="22" customHeight="1">
+      <c r="A27" s="8" t="inlineStr">
         <is>
           <t>Twilio Speech-to-Text, $ per minute</t>
         </is>
       </c>
-      <c r="B27" s="19" t="n">
+      <c r="B27" s="24" t="n">
         <v>0.02</v>
       </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="9" t="inlineStr">
+      <c r="C27" s="21" t="n"/>
+      <c r="D27" s="21" t="n"/>
+      <c r="E27" s="21" t="n"/>
+    </row>
+    <row r="28" ht="22" customHeight="1">
+      <c r="A28" s="11" t="inlineStr">
         <is>
           <t>Claude Haiku, flat $ per call</t>
         </is>
       </c>
-      <c r="B28" s="19" t="n">
+      <c r="B28" s="22" t="n">
         <v>0.002</v>
       </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="9" t="inlineStr">
+      <c r="C28" s="23" t="n"/>
+      <c r="D28" s="23" t="n"/>
+      <c r="E28" s="23" t="n"/>
+    </row>
+    <row r="29" ht="22" customHeight="1">
+      <c r="A29" s="8" t="inlineStr">
         <is>
           <t>Cheap Text-to-Speech, flat $ per call</t>
         </is>
       </c>
-      <c r="B29" s="19" t="n">
+      <c r="B29" s="24" t="n">
         <v>0.001</v>
       </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="9" t="inlineStr">
+      <c r="C29" s="21" t="n"/>
+      <c r="D29" s="21" t="n"/>
+      <c r="E29" s="21" t="n"/>
+    </row>
+    <row r="30" ht="22" customHeight="1">
+      <c r="A30" s="11" t="inlineStr">
         <is>
           <t>ElevenLabs, $ per minute</t>
         </is>
       </c>
-      <c r="B30" s="19" t="n">
+      <c r="B30" s="22" t="n">
         <v>0.1</v>
       </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="9" t="inlineStr">
+      <c r="C30" s="23" t="n"/>
+      <c r="D30" s="23" t="n"/>
+      <c r="E30" s="23" t="n"/>
+    </row>
+    <row r="31" ht="22" customHeight="1">
+      <c r="A31" s="8" t="inlineStr">
         <is>
           <t>Claude Sonnet 4.6, $ per minute</t>
         </is>
       </c>
-      <c r="B31" s="19" t="n">
+      <c r="B31" s="24" t="n">
         <v>0.024</v>
       </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="9" t="inlineStr">
+      <c r="C31" s="21" t="n"/>
+      <c r="D31" s="21" t="n"/>
+      <c r="E31" s="21" t="n"/>
+    </row>
+    <row r="32" ht="22" customHeight="1">
+      <c r="A32" s="11" t="inlineStr">
         <is>
           <t>Railway server, flat $ per call</t>
         </is>
       </c>
-      <c r="B32" s="19" t="n">
+      <c r="B32" s="22" t="n">
         <v>0.001</v>
       </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="9" t="inlineStr">
+      <c r="C32" s="23" t="n"/>
+      <c r="D32" s="23" t="n"/>
+      <c r="E32" s="23" t="n"/>
+    </row>
+    <row r="33" ht="22" customHeight="1">
+      <c r="A33" s="8" t="inlineStr">
         <is>
           <t>Twilio number, flat $ per call</t>
         </is>
       </c>
-      <c r="B33" s="19" t="n">
+      <c r="B33" s="24" t="n">
         <v>0.001</v>
       </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="9" t="inlineStr">
+      <c r="C33" s="21" t="n"/>
+      <c r="D33" s="21" t="n"/>
+      <c r="E33" s="21" t="n"/>
+    </row>
+    <row r="34" ht="22" customHeight="1">
+      <c r="A34" s="11" t="inlineStr">
         <is>
           <t>Selling price per check</t>
         </is>
       </c>
-      <c r="B34" s="20" t="n">
+      <c r="B34" s="25" t="n">
         <v>0.25</v>
       </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="9" t="inlineStr">
-        <is>
-          <t>(helper) Is Voice = 1</t>
-        </is>
-      </c>
-      <c r="B35" s="18">
+      <c r="C34" s="23" t="n"/>
+      <c r="D34" s="23" t="n"/>
+      <c r="E34" s="23" t="n"/>
+    </row>
+    <row r="35" ht="22" customHeight="1">
+      <c r="A35" s="8" t="inlineStr">
+        <is>
+          <t>(helper) Is Voice</t>
+        </is>
+      </c>
+      <c r="B35" s="20">
         <f>IF(B2="VOICE (voice only tree - CVS)",1,0)</f>
         <v/>
       </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="9" t="inlineStr">
-        <is>
-          <t>(helper) Is Keypad = 1</t>
-        </is>
-      </c>
-      <c r="B36" s="18">
+      <c r="C35" s="21" t="n"/>
+      <c r="D35" s="21" t="n"/>
+      <c r="E35" s="21" t="n"/>
+    </row>
+    <row r="36" ht="22" customHeight="1">
+      <c r="A36" s="11" t="inlineStr">
+        <is>
+          <t>(helper) Is Keypad</t>
+        </is>
+      </c>
+      <c r="B36" s="26">
         <f>IF(B2="KEYPAD (no voice tree - Walgreens)",1,0)</f>
         <v/>
       </c>
+      <c r="C36" s="23" t="n"/>
+      <c r="D36" s="23" t="n"/>
+      <c r="E36" s="23" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="12">
+  <mergeCells count="13">
     <mergeCell ref="A20:B20"/>
     <mergeCell ref="A12:E12"/>
     <mergeCell ref="A21:B21"/>
     <mergeCell ref="A15:B15"/>
+    <mergeCell ref="B4:E4"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A16:E16"/>
     <mergeCell ref="A24:E24"/>
-    <mergeCell ref="A16:E16"/>
     <mergeCell ref="A11:B11"/>
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="B2:E2"/>
+    <mergeCell ref="A5:E5"/>
     <mergeCell ref="A6:E6"/>
     <mergeCell ref="A22:B22"/>
-    <mergeCell ref="A3:E3"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="B2" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="B4" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"DIRECT CALL (no trees - Ross),KEYPAD (no voice tree - Walgreens),VOICE (voice only tree - CVS)"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>